<commit_message>
Stress test (app, report, workbook); plans use the 2026 rules by default; report fits its pages; workbook v3.0 with stress sheets
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhUEAkgdki1q9EpFqaquGU
</commit_message>
<xml_diff>
--- a/deliverables/LifeGoals-Calculators-Reference.xlsx
+++ b/deliverables/LifeGoals-Calculators-Reference.xlsx
@@ -4873,7 +4873,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="B120" t="inlineStr">
+      <c r="B120" s="170" t="inlineStr">
         <is>
           <t>Plan holdings</t>
         </is>
@@ -4885,7 +4885,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="B121" t="inlineStr">
+      <c r="B121" s="170" t="inlineStr">
         <is>
           <t>Funding order</t>
         </is>
@@ -4897,7 +4897,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="B122" t="inlineStr">
+      <c r="B122" s="170" t="inlineStr">
         <is>
           <t>Home and policies</t>
         </is>
@@ -4909,7 +4909,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="B123" t="inlineStr">
+      <c r="B123" s="170" t="inlineStr">
         <is>
           <t>Two assumptions only the 2026 workbook has</t>
         </is>
@@ -4921,7 +4921,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="B124" t="inlineStr">
+      <c r="B124" s="170" t="inlineStr">
         <is>
           <t>Checked against the app</t>
         </is>
@@ -4940,240 +4940,240 @@
       </c>
     </row>
     <row r="127">
-      <c r="B127" t="inlineStr">
+      <c r="B127" s="170" t="inlineStr">
         <is>
           <t>In_savings / Has_savings</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
+      <c r="C127" s="170" t="inlineStr">
         <is>
           <t>Savings accounts   [S.fin.savings]</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="B128" t="inlineStr">
+      <c r="B128" s="170" t="inlineStr">
         <is>
           <t>In_otherAssets / Has_otherAssets</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
+      <c r="C128" s="170" t="inlineStr">
         <is>
           <t>Other assets you would sell if needed   [S.fin.otherAssets]</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="B129" t="inlineStr">
+      <c r="B129" s="170" t="inlineStr">
         <is>
           <t>In_altInv / Has_altInv</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
+      <c r="C129" s="170" t="inlineStr">
         <is>
           <t>Alternative investments   [S.fin.altInv]</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="B130" t="inlineStr">
+      <c r="B130" s="170" t="inlineStr">
         <is>
           <t>In_invCost / Has_invCost</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
+      <c r="C130" s="170" t="inlineStr">
         <is>
           <t>What you paid for your investments   [S.fin.invCost, blank = unknown]</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="B131" t="inlineStr">
+      <c r="B131" s="170" t="inlineStr">
         <is>
           <t>In_invYears / Has_invYears</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
+      <c r="C131" s="170" t="inlineStr">
         <is>
           <t>Years you have held your investments   [S.fin.invYears]</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="B132" t="inlineStr">
+      <c r="B132" s="170" t="inlineStr">
         <is>
           <t>In_othCost / Has_othCost</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr">
+      <c r="C132" s="170" t="inlineStr">
         <is>
           <t>What you paid for other assets   [S.fin.othCost]</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="B133" t="inlineStr">
+      <c r="B133" s="170" t="inlineStr">
         <is>
           <t>In_altCost / Has_altCost</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
+      <c r="C133" s="170" t="inlineStr">
         <is>
           <t>What you paid for alternative investments   [S.fin.altCost]</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="B134" t="inlineStr">
+      <c r="B134" s="170" t="inlineStr">
         <is>
           <t>In_capLoss / Has_capLoss</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
+      <c r="C134" s="170" t="inlineStr">
         <is>
           <t>Capital losses you can use   [S.fin.capLoss]</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="B135" t="inlineStr">
+      <c r="B135" s="170" t="inlineStr">
         <is>
           <t>In_assetsJoint / Has_assetsJoint</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
+      <c r="C135" s="170" t="inlineStr">
         <is>
           <t>Assets owned with your partner   [S.fin.assetsJoint]</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="B136" t="inlineStr">
+      <c r="B136" s="170" t="inlineStr">
         <is>
           <t>In_homeUse / Has_homeUse</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
+      <c r="C136" s="170" t="inlineStr">
         <is>
           <t>Would you use your home to fund your plan   [S.fin.homeUse]</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="B137" t="inlineStr">
+      <c r="B137" s="170" t="inlineStr">
         <is>
           <t>In_downAge / Has_downAge</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
+      <c r="C137" s="170" t="inlineStr">
         <is>
           <t>Age you would downsize   [S.fin.downAge]</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="B138" t="inlineStr">
+      <c r="B138" s="170" t="inlineStr">
         <is>
           <t>In_downValue / Has_downValue</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
+      <c r="C138" s="170" t="inlineStr">
         <is>
           <t>Value of the smaller home   [S.fin.downValue]</t>
         </is>
       </c>
     </row>
     <row r="139">
-      <c r="B139" t="inlineStr">
+      <c r="B139" s="170" t="inlineStr">
         <is>
           <t>In_polLump / Has_polLump</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
+      <c r="C139" s="170" t="inlineStr">
         <is>
           <t>Policy lump sum   [S.fin.polLump]</t>
         </is>
       </c>
     </row>
     <row r="140">
-      <c r="B140" t="inlineStr">
+      <c r="B140" s="170" t="inlineStr">
         <is>
           <t>In_polLumpAge / Has_polLumpAge</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
+      <c r="C140" s="170" t="inlineStr">
         <is>
           <t>Age the lump sum is paid   [S.fin.polLumpAge]</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="B141" t="inlineStr">
+      <c r="B141" s="170" t="inlineStr">
         <is>
           <t>In_polInc / Has_polInc</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
+      <c r="C141" s="170" t="inlineStr">
         <is>
           <t>Policy or annuity income a year   [S.fin.polInc]</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="B142" t="inlineStr">
+      <c r="B142" s="170" t="inlineStr">
         <is>
           <t>In_polIncAge / Has_polIncAge</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr">
+      <c r="C142" s="170" t="inlineStr">
         <is>
           <t>Age the income starts   [S.fin.polIncAge]</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="B143" t="inlineStr">
+      <c r="B143" s="170" t="inlineStr">
         <is>
           <t>In_safetyWanted / Has_safetyWanted</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr">
+      <c r="C143" s="170" t="inlineStr">
         <is>
           <t>Asked for an Emergency fund goal   [S.safetyWanted]</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="B144" t="inlineStr">
+      <c r="B144" s="170" t="inlineStr">
         <is>
           <t>In_safetyOff / Has_safetyOff</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
+      <c r="C144" s="170" t="inlineStr">
         <is>
           <t>Removed the Emergency fund goal   [S.safetyOff]</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="B145" t="inlineStr">
+      <c r="B145" s="170" t="inlineStr">
         <is>
           <t>In_a_invWrapper / Has_a_invWrapper</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr">
+      <c r="C145" s="170" t="inlineStr">
         <is>
           <t>Investments held as funds (fund) or shares   [S.asm.invWrapper]</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="B146" t="inlineStr">
+      <c r="B146" s="170" t="inlineStr">
         <is>
           <t>In_a_cgtGain / Has_a_cgtGain</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
+      <c r="C146" s="170" t="inlineStr">
         <is>
           <t>Gain share when no cost is given   [S.asm.cgtGain]</t>
         </is>
@@ -5193,7 +5193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:H117"/>
+  <dimension ref="A1:H118"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2" customWidth="1" style="170" min="1" max="1"/>
@@ -9047,6 +9047,18 @@
       </c>
       <c r="D117" s="170" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Stress test (Plan stress test sheet)</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>A side run of the plan: in the year before the retirement age (this year if already retired) pension pots and invested money (invested share of spare money, invested goal pots, investments, alternative investments) fall by ST_Fall (20%) instead of growing. Cash, savings accounts, the emergency fund and price-linked assets do not fall. Copies of the engine sheets (Stress pay &amp; tax, holdings, goals, cashflow, hidden at the end) differ only in that growth. Outputs: ST1..ST22_Pct, ST_RunOutAge (and base), ST_PotAtRet (and base), ST_Line. Matches the prototype stressInfo().</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -22027,8 +22039,8 @@
     <mergeCell ref="D117:E117"/>
     <mergeCell ref="D92:E92"/>
     <mergeCell ref="B8:E8"/>
+    <mergeCell ref="D130:E130"/>
     <mergeCell ref="D94:E94"/>
-    <mergeCell ref="D130:E130"/>
     <mergeCell ref="D82:E82"/>
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="D98:E98"/>

</xml_diff>